<commit_message>
Plan for lab comparative experiments added
</commit_message>
<xml_diff>
--- a/Field-trails/Cattle-Slurry 2025-10-28/slurry pH at aplication.xlsx
+++ b/Field-trails/Cattle-Slurry 2025-10-28/slurry pH at aplication.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Fall field trails\Cattle_slurry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\Cattle-Slurry 2025-10-28\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C707172-8020-46B3-A85A-5261D36909FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B523C3-E3AA-4125-8995-6728E514DD21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pH at aplication" sheetId="1" r:id="rId1"/>
@@ -174,10 +174,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,7 +443,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.88671875" customWidth="1"/>
     <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>